<commit_message>
FC design v0.5 corrected
</commit_message>
<xml_diff>
--- a/hardware/Component-Library.xlsx
+++ b/hardware/Component-Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andgui\Projects\Flight-Controller\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6B655A-0DD2-4B91-BD25-694AB52E57A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB37A29-BE1B-4E0D-8B4C-7765E2429F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="2115" windowWidth="24990" windowHeight="13080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3330" yWindow="2310" windowWidth="24990" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ICs" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
changing USB ESD IC (v0.8)
</commit_message>
<xml_diff>
--- a/hardware/Component-Library.xlsx
+++ b/hardware/Component-Library.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andgui\Projects\Flight-Controller\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49150026-AC8E-4976-967B-960544612CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5062E773-6FCD-4CE2-87A4-3C7E1B9CE98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4110" yWindow="1275" windowWidth="24990" windowHeight="13080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ICs" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="resources" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="232">
   <si>
     <t>Category</t>
   </si>
@@ -548,9 +549,6 @@
     <t>DigiKey-USBLC6</t>
   </si>
   <si>
-    <t>TVS DIODE 5.25VWM 17VC</t>
-  </si>
-  <si>
     <t>JLCPCB-TPS62130</t>
   </si>
   <si>
@@ -708,6 +706,27 @@
   </si>
   <si>
     <t>..\resources\datasheets\ESD\USBLC6-2-datasheet.pdf</t>
+  </si>
+  <si>
+    <t>TPD2EUSB30ADRTR</t>
+  </si>
+  <si>
+    <t>SOT-23-3 Variant</t>
+  </si>
+  <si>
+    <t>For self powered devices TVS DIODE 5.25VWM 17VC</t>
+  </si>
+  <si>
+    <t>..\resources\datasheets\ESD\tpd2eusb30a.pdf</t>
+  </si>
+  <si>
+    <t>DigiKey-TPD2EUSB30A</t>
+  </si>
+  <si>
+    <t>JLCPCBs-TPD2EUSB30A</t>
+  </si>
+  <si>
+    <t>TVS DIODE 3.6VWM 8VC</t>
   </si>
 </sst>
 </file>
@@ -1610,10 +1629,10 @@
         <v>5</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="3:11" ht="30" x14ac:dyDescent="0.25">
@@ -1638,7 +1657,7 @@
       </c>
       <c r="J6" s="8"/>
       <c r="K6" s="27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="3:11" ht="30" x14ac:dyDescent="0.25">
@@ -1647,10 +1666,10 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>12</v>
@@ -1662,10 +1681,10 @@
         <v>6</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="3:11" x14ac:dyDescent="0.25">
@@ -1691,10 +1710,10 @@
         <v>5</v>
       </c>
       <c r="J8" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="K8" s="27" t="s">
         <v>176</v>
-      </c>
-      <c r="K8" s="27" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="9" spans="3:11" x14ac:dyDescent="0.25">
@@ -1766,10 +1785,10 @@
         <v>5</v>
       </c>
       <c r="J11" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="K11" s="27" t="s">
         <v>178</v>
-      </c>
-      <c r="K11" s="27" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="12" spans="3:11" x14ac:dyDescent="0.25">
@@ -1811,7 +1830,7 @@
         <v>33</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="3:11" x14ac:dyDescent="0.25">
@@ -1889,72 +1908,72 @@
     </row>
     <row r="18" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C18" s="53" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E18" t="s">
         <v>63</v>
       </c>
       <c r="F18" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="G18" s="13" t="s">
         <v>198</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>199</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>5</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="35" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K18" s="27" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C19" s="55"/>
       <c r="D19" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>45</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I19" s="6"/>
       <c r="K19" s="27" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C20" s="51"/>
       <c r="D20" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="31"/>
       <c r="G20" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="35" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K20" s="27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="3:11" x14ac:dyDescent="0.25">
@@ -1978,7 +1997,7 @@
         <v>6</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K21" s="27" t="s">
         <v>65</v>
@@ -2122,14 +2141,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{670BDE95-32D1-49FD-9C5A-9CBB1FAE7FE3}">
-  <dimension ref="B3:J24"/>
+  <dimension ref="B3:J25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.5703125" style="24" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="49.5703125" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
     <col min="8" max="8" width="9.5703125" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
@@ -2205,7 +2224,7 @@
         <v>5</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>43</v>
@@ -2374,7 +2393,7 @@
       </c>
       <c r="E12" s="29"/>
       <c r="F12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>5</v>
@@ -2412,71 +2431,71 @@
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="38"/>
       <c r="C15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>50</v>
       </c>
       <c r="E15" s="29"/>
       <c r="F15" t="s">
+        <v>201</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="J15" s="11" t="s">
         <v>202</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="38"/>
       <c r="C16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E16" s="29"/>
       <c r="F16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="C17" t="s">
         <v>210</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>212</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>213</v>
+      </c>
+      <c r="F17" t="s">
         <v>211</v>
       </c>
-      <c r="D17" t="s">
-        <v>213</v>
-      </c>
-      <c r="E17" s="28" t="s">
+      <c r="G17" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="J17" s="11" t="s">
         <v>214</v>
-      </c>
-      <c r="F17" t="s">
-        <v>212</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
@@ -2484,160 +2503,184 @@
         <v>107</v>
       </c>
       <c r="C18" t="s">
-        <v>168</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>169</v>
+        <v>225</v>
+      </c>
+      <c r="D18" t="s">
+        <v>226</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F18" t="s">
-        <v>172</v>
+        <v>231</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>5</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>171</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="38"/>
       <c r="C19" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" t="s">
-        <v>110</v>
+        <v>168</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>169</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>151</v>
+        <v>224</v>
       </c>
       <c r="F19" t="s">
-        <v>109</v>
+        <v>227</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>112</v>
+        <v>170</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>111</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="38"/>
       <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>110</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="F20" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="J20" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="38"/>
+      <c r="C21" t="s">
         <v>113</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D21" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E21" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F21" t="s">
         <v>114</v>
       </c>
-      <c r="G20" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I20" s="11" t="s">
+      <c r="G21" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I21" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J21" s="11" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B21" s="9" t="s">
+    <row r="22" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B22" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>120</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E22" s="28" t="s">
         <v>153</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="F22" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I21" s="11" t="s">
+      <c r="G22" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I22" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J22" s="11" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="38" t="s">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>157</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D23" t="s">
         <v>158</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E23" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F23" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J22" s="11" t="s">
+      <c r="J23" s="11" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="38"/>
-      <c r="C23" t="s">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="38"/>
+      <c r="C24" t="s">
         <v>162</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D24" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F24" t="s">
         <v>166</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I23" s="11" t="s">
+      <c r="G24" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I24" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="J23" s="11" t="s">
+      <c r="J24" s="11" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>217</v>
+      </c>
+      <c r="C25" t="s">
         <v>218</v>
       </c>
-      <c r="C24" t="s">
-        <v>219</v>
-      </c>
-      <c r="F24" s="25"/>
+      <c r="F25" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="D3:F3"/>
@@ -2646,10 +2689,10 @@
     <mergeCell ref="B5:B8"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="B18:B21"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G5:H8 G9:G23">
+  <conditionalFormatting sqref="G5:H8 G9:G24">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"no"</formula>
     </cfRule>
@@ -2658,7 +2701,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:H8 G9:G23" xr:uid="{16E70C10-E0D8-4840-AEA1-7AA8C21C6052}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:H8 G9:G24" xr:uid="{16E70C10-E0D8-4840-AEA1-7AA8C21C6052}">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2681,24 +2724,24 @@
     <hyperlink ref="E11" r:id="rId16" xr:uid="{2F7D2E1C-572A-40A6-A537-AE8A71A84B92}"/>
     <hyperlink ref="J10" r:id="rId17" xr:uid="{078108F6-3106-4427-8212-509361A32B23}"/>
     <hyperlink ref="I12" r:id="rId18" xr:uid="{4B806AB2-B5DE-4DCB-AC21-E51C140EAA6F}"/>
-    <hyperlink ref="E19" r:id="rId19" xr:uid="{B84D1D11-4839-4507-866F-3DB821FC7223}"/>
-    <hyperlink ref="J19" r:id="rId20" xr:uid="{45063706-F8DD-4586-B532-1AF1FFE4D222}"/>
-    <hyperlink ref="I19" r:id="rId21" xr:uid="{D608BFA7-83BF-4D1F-82B5-5A142FAD149B}"/>
-    <hyperlink ref="E20" r:id="rId22" xr:uid="{4E4966D7-5D9C-457C-875C-140C265069B0}"/>
-    <hyperlink ref="J20" r:id="rId23" xr:uid="{2C2D94D1-BDF7-426D-8EFB-1C4770F313BB}"/>
-    <hyperlink ref="I20" r:id="rId24" xr:uid="{E1BC785D-5519-4540-A6B1-C307CDC6A748}"/>
-    <hyperlink ref="J21" r:id="rId25" xr:uid="{FE26BA89-AE20-400E-A204-A1D51563DF5F}"/>
-    <hyperlink ref="I21" r:id="rId26" xr:uid="{4380D086-6180-45C1-9F84-52BBDD26E612}"/>
-    <hyperlink ref="E21" r:id="rId27" xr:uid="{F01D8885-58E5-4152-89A6-1D3EFB41E879}"/>
+    <hyperlink ref="E20" r:id="rId19" xr:uid="{B84D1D11-4839-4507-866F-3DB821FC7223}"/>
+    <hyperlink ref="J20" r:id="rId20" xr:uid="{45063706-F8DD-4586-B532-1AF1FFE4D222}"/>
+    <hyperlink ref="I20" r:id="rId21" xr:uid="{D608BFA7-83BF-4D1F-82B5-5A142FAD149B}"/>
+    <hyperlink ref="E21" r:id="rId22" xr:uid="{4E4966D7-5D9C-457C-875C-140C265069B0}"/>
+    <hyperlink ref="J21" r:id="rId23" xr:uid="{2C2D94D1-BDF7-426D-8EFB-1C4770F313BB}"/>
+    <hyperlink ref="I21" r:id="rId24" xr:uid="{E1BC785D-5519-4540-A6B1-C307CDC6A748}"/>
+    <hyperlink ref="J22" r:id="rId25" xr:uid="{FE26BA89-AE20-400E-A204-A1D51563DF5F}"/>
+    <hyperlink ref="I22" r:id="rId26" xr:uid="{4380D086-6180-45C1-9F84-52BBDD26E612}"/>
+    <hyperlink ref="E22" r:id="rId27" xr:uid="{F01D8885-58E5-4152-89A6-1D3EFB41E879}"/>
     <hyperlink ref="E8" r:id="rId28" xr:uid="{A66C6588-B22D-48F2-A4EC-7D0E46AD60F3}"/>
-    <hyperlink ref="E22" r:id="rId29" xr:uid="{B51B99C6-1910-491D-81A6-E411A3AE7908}"/>
-    <hyperlink ref="J22" r:id="rId30" xr:uid="{D4B2B14F-519C-40B0-AC9E-652A1615F7B2}"/>
-    <hyperlink ref="D23" r:id="rId31" display="https://www.digikey.com.au/en/products/filter/transistors/fets-mosfets/single-fets-mosfets/3-smd-sot-23-3-variant/278?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAJgAYWBWWTkAXQIAHMlBABlSgEtiAcxABfRUA" xr:uid="{427053F7-D1E6-4161-A03E-357918EA99BE}"/>
-    <hyperlink ref="J23" r:id="rId32" xr:uid="{A8094415-9801-4570-832C-C2DE47B8EED0}"/>
-    <hyperlink ref="E23" r:id="rId33" xr:uid="{3300C72A-8FEE-49E7-9F94-26680825DC19}"/>
-    <hyperlink ref="I23" r:id="rId34" xr:uid="{12A90CC8-ABE8-4E1C-B7E9-A039C71E7360}"/>
-    <hyperlink ref="I18" r:id="rId35" xr:uid="{9333B8F5-7A23-4277-901C-C048FA77551E}"/>
-    <hyperlink ref="J18" r:id="rId36" xr:uid="{1F9C453E-8146-4ABB-B0D8-ADC0F74BDFDD}"/>
+    <hyperlink ref="E23" r:id="rId29" xr:uid="{B51B99C6-1910-491D-81A6-E411A3AE7908}"/>
+    <hyperlink ref="J23" r:id="rId30" xr:uid="{D4B2B14F-519C-40B0-AC9E-652A1615F7B2}"/>
+    <hyperlink ref="D24" r:id="rId31" display="https://www.digikey.com.au/en/products/filter/transistors/fets-mosfets/single-fets-mosfets/3-smd-sot-23-3-variant/278?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAJgAYWBWWTkAXQIAHMlBABlSgEtiAcxABfRUA" xr:uid="{427053F7-D1E6-4161-A03E-357918EA99BE}"/>
+    <hyperlink ref="J24" r:id="rId32" xr:uid="{A8094415-9801-4570-832C-C2DE47B8EED0}"/>
+    <hyperlink ref="E24" r:id="rId33" xr:uid="{3300C72A-8FEE-49E7-9F94-26680825DC19}"/>
+    <hyperlink ref="I24" r:id="rId34" xr:uid="{12A90CC8-ABE8-4E1C-B7E9-A039C71E7360}"/>
+    <hyperlink ref="I19" r:id="rId35" xr:uid="{9333B8F5-7A23-4277-901C-C048FA77551E}"/>
+    <hyperlink ref="J19" r:id="rId36" xr:uid="{1F9C453E-8146-4ABB-B0D8-ADC0F74BDFDD}"/>
     <hyperlink ref="I5" r:id="rId37" xr:uid="{C4E7B030-4D65-46DD-B8CD-32E254C3E9BC}"/>
     <hyperlink ref="J15" r:id="rId38" xr:uid="{A2D551F1-2E4B-4156-B207-EC4CE5E7FC8B}"/>
     <hyperlink ref="I15" r:id="rId39" xr:uid="{CFFF530B-2773-42DF-90C4-202FCF4E4B7A}"/>
@@ -2707,7 +2750,10 @@
     <hyperlink ref="E17" r:id="rId42" xr:uid="{B36D8326-BCC3-4582-9004-FC7C01706DCB}"/>
     <hyperlink ref="J17" r:id="rId43" xr:uid="{30D79133-F02A-453B-AB7E-C10F953868B8}"/>
     <hyperlink ref="I17" r:id="rId44" xr:uid="{828B557D-59E0-4E1C-B749-5FDFC6187973}"/>
-    <hyperlink ref="E18" r:id="rId45" xr:uid="{17EC64C7-81E0-4782-83D8-B81B200B35F9}"/>
+    <hyperlink ref="E19" r:id="rId45" xr:uid="{17EC64C7-81E0-4782-83D8-B81B200B35F9}"/>
+    <hyperlink ref="E18" r:id="rId46" xr:uid="{CC3FB449-A5FB-45C6-B6EE-0F3148FD427A}"/>
+    <hyperlink ref="J18" r:id="rId47" xr:uid="{03F4CC3D-F7CE-4EE4-A6FB-D01FDB9B37EE}"/>
+    <hyperlink ref="I18" r:id="rId48" xr:uid="{D880243D-A403-4FCF-9CC6-F7F21A6C9531}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -2801,7 +2847,7 @@
         <v>5</v>
       </c>
       <c r="I4" s="21" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J4" s="21" t="s">
         <v>58</v>
@@ -2812,13 +2858,13 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="6" t="s">
@@ -2828,10 +2874,10 @@
         <v>5</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Component library fully complete
</commit_message>
<xml_diff>
--- a/hardware/Component-Library.xlsx
+++ b/hardware/Component-Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\andgui\Projects\Flight-Controller\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30252389-2C1E-4A48-B221-142DFB81C6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78862944-C232-4D15-8510-0599A086F488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="1095" windowWidth="24990" windowHeight="13080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ICs" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="312">
   <si>
     <t>Category</t>
   </si>
@@ -941,6 +941,42 @@
   </si>
   <si>
     <t>JLCPCB-X322516M</t>
+  </si>
+  <si>
+    <t>LTVS16H5.0T5G</t>
+  </si>
+  <si>
+    <t>DFN1610-2</t>
+  </si>
+  <si>
+    <t>..\resources\datasheets\ESD\LTVS16H5.pdf</t>
+  </si>
+  <si>
+    <t>100A@8/20us 2uA 5V 7.8V 8.5V 15V 800pF ESD Unidirectional</t>
+  </si>
+  <si>
+    <t>JLCPCB-LTVS16H5</t>
+  </si>
+  <si>
+    <t>KT-0603R</t>
+  </si>
+  <si>
+    <t>..\resources\datasheets\LED\KT-0603R.pdf</t>
+  </si>
+  <si>
+    <t>JLCPCB-KT0603R</t>
+  </si>
+  <si>
+    <t>KT-0603W</t>
+  </si>
+  <si>
+    <t>..\resources\datasheets\LED\KT-0603W.pdf</t>
+  </si>
+  <si>
+    <t>White yellow LED</t>
+  </si>
+  <si>
+    <t>JLCPCB-KT0603W</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1227,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -1246,84 +1282,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -1332,15 +1290,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
@@ -1357,18 +1309,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1389,9 +1330,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1404,15 +1342,111 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1868,29 +1902,29 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="43" t="s">
+      <c r="E2" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="44"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="31" t="s">
+      <c r="F2" s="89"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="32"/>
-      <c r="J2" s="31" t="s">
+      <c r="I2" s="74"/>
+      <c r="J2" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="32"/>
+      <c r="K2" s="74"/>
     </row>
     <row r="3" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
       <c r="E3" s="13" t="s">
         <v>37</v>
       </c>
@@ -1914,32 +1948,32 @@
       </c>
     </row>
     <row r="4" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="85" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="42"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="86"/>
+      <c r="H4" s="86"/>
+      <c r="I4" s="86"/>
+      <c r="J4" s="86"/>
+      <c r="K4" s="87"/>
     </row>
     <row r="5" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="85" t="s">
+      <c r="D5" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="69" t="s">
+      <c r="E5" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="G5" s="86" t="s">
+      <c r="G5" s="49" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="6" t="s">
@@ -1956,7 +1990,7 @@
       </c>
     </row>
     <row r="6" spans="3:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="C6" s="47"/>
+      <c r="C6" s="72"/>
       <c r="D6" s="16" t="s">
         <v>4</v>
       </c>
@@ -1981,17 +2015,17 @@
       </c>
     </row>
     <row r="7" spans="3:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="C7" s="47"/>
-      <c r="D7" s="85" t="s">
+      <c r="C7" s="72"/>
+      <c r="D7" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="69" t="s">
+      <c r="E7" s="39" t="s">
         <v>217</v>
       </c>
-      <c r="F7" s="71" t="s">
+      <c r="F7" s="41" t="s">
         <v>216</v>
       </c>
-      <c r="G7" s="88" t="s">
+      <c r="G7" s="51" t="s">
         <v>12</v>
       </c>
       <c r="H7" t="s">
@@ -2008,19 +2042,19 @@
       </c>
     </row>
     <row r="8" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="85" t="s">
+      <c r="D8" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="69" t="s">
+      <c r="E8" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="71" t="s">
+      <c r="F8" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="86" t="s">
+      <c r="G8" s="49" t="s">
         <v>19</v>
       </c>
       <c r="H8" s="6" t="s">
@@ -2037,7 +2071,7 @@
       </c>
     </row>
     <row r="9" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C9" s="47"/>
+      <c r="C9" s="72"/>
       <c r="D9" s="16" t="s">
         <v>14</v>
       </c>
@@ -2060,7 +2094,7 @@
       <c r="K9" s="1"/>
     </row>
     <row r="10" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C10" s="47" t="s">
+      <c r="C10" s="72" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -2085,17 +2119,17 @@
       <c r="K10" s="1"/>
     </row>
     <row r="11" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C11" s="48"/>
-      <c r="D11" s="85" t="s">
+      <c r="C11" s="92"/>
+      <c r="D11" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="86" t="s">
+      <c r="E11" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="87" t="s">
+      <c r="F11" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="G11" s="69" t="s">
+      <c r="G11" s="39" t="s">
         <v>44</v>
       </c>
       <c r="H11" t="s">
@@ -2112,32 +2146,32 @@
       </c>
     </row>
     <row r="12" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="82" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="39"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="83"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="83"/>
+      <c r="K12" s="84"/>
     </row>
     <row r="13" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="86" t="s">
+      <c r="D13" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="69" t="s">
+      <c r="E13" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="71" t="s">
+      <c r="F13" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="G13" s="69" t="s">
+      <c r="G13" s="39" t="s">
         <v>44</v>
       </c>
       <c r="H13" s="6" t="s">
@@ -2154,7 +2188,7 @@
       </c>
     </row>
     <row r="14" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C14" s="49"/>
+      <c r="C14" s="93"/>
       <c r="D14" s="4" t="s">
         <v>22</v>
       </c>
@@ -2169,7 +2203,7 @@
       <c r="K14" s="1"/>
     </row>
     <row r="15" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C15" s="49"/>
+      <c r="C15" s="93"/>
       <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
@@ -2187,32 +2221,32 @@
       <c r="K15" s="1"/>
     </row>
     <row r="16" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="82" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="39"/>
+      <c r="D16" s="83"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="83"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="83"/>
+      <c r="K16" s="84"/>
     </row>
     <row r="17" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C17" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="94" t="s">
+      <c r="D17" s="56" t="s">
         <v>293</v>
       </c>
-      <c r="E17" s="73" t="s">
+      <c r="E17" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="95" t="s">
+      <c r="F17" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="G17" s="73" t="s">
+      <c r="G17" s="43" t="s">
         <v>59</v>
       </c>
       <c r="H17" s="6" t="s">
@@ -2227,19 +2261,19 @@
       </c>
     </row>
     <row r="18" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="92" t="s">
         <v>181</v>
       </c>
-      <c r="D18" s="94" t="s">
+      <c r="D18" s="56" t="s">
         <v>190</v>
       </c>
-      <c r="E18" s="69" t="s">
+      <c r="E18" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="F18" s="95" t="s">
+      <c r="F18" s="57" t="s">
         <v>193</v>
       </c>
-      <c r="G18" s="73" t="s">
+      <c r="G18" s="43" t="s">
         <v>194</v>
       </c>
       <c r="H18" s="6" t="s">
@@ -2254,7 +2288,7 @@
       </c>
     </row>
     <row r="19" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C19" s="50"/>
+      <c r="C19" s="94"/>
       <c r="D19" s="2" t="s">
         <v>185</v>
       </c>
@@ -2276,7 +2310,7 @@
       </c>
     </row>
     <row r="20" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C20" s="46"/>
+      <c r="C20" s="91"/>
       <c r="D20" s="2" t="s">
         <v>182</v>
       </c>
@@ -2300,16 +2334,16 @@
       <c r="C21" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="94" t="s">
+      <c r="D21" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="96" t="s">
+      <c r="E21" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="95" t="s">
+      <c r="F21" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="G21" s="97"/>
+      <c r="G21" s="59"/>
       <c r="H21" s="6" t="s">
         <v>5</v>
       </c>
@@ -2324,32 +2358,32 @@
       </c>
     </row>
     <row r="22" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="79" t="s">
         <v>120</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="79"/>
+      <c r="I22" s="79"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="79"/>
     </row>
     <row r="23" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="80" t="s">
         <v>121</v>
       </c>
-      <c r="D23" s="69" t="s">
+      <c r="D23" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="E23" s="69" t="s">
+      <c r="E23" s="39" t="s">
         <v>123</v>
       </c>
-      <c r="F23" s="71" t="s">
+      <c r="F23" s="41" t="s">
         <v>139</v>
       </c>
-      <c r="G23" s="69" t="s">
+      <c r="G23" s="39" t="s">
         <v>125</v>
       </c>
       <c r="H23" s="6" t="s">
@@ -2363,7 +2397,7 @@
       </c>
     </row>
     <row r="24" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C24" s="30"/>
+      <c r="C24" s="81"/>
       <c r="D24" t="s">
         <v>127</v>
       </c>
@@ -2461,7 +2495,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{670BDE95-32D1-49FD-9C5A-9CBB1FAE7FE3}">
-  <dimension ref="B3:J46"/>
+  <dimension ref="B3:J49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
@@ -2476,29 +2510,29 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="33"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="31" t="s">
+      <c r="E3" s="75"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="32"/>
-      <c r="I3" s="31" t="s">
+      <c r="H3" s="74"/>
+      <c r="I3" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="32"/>
+      <c r="J3" s="74"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="20" t="s">
         <v>37</v>
       </c>
@@ -2522,19 +2556,19 @@
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="C5" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="70" t="s">
+      <c r="D5" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="71" t="s">
+      <c r="E5" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="F5" s="69" t="s">
+      <c r="F5" s="39" t="s">
         <v>36</v>
       </c>
       <c r="G5" s="6" t="s">
@@ -2551,887 +2585,956 @@
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="47"/>
-      <c r="C6" t="s">
+      <c r="B6" s="72"/>
+      <c r="C6" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="41" t="s">
+        <v>306</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="72"/>
+      <c r="C7" s="39" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="E7" s="41" t="s">
+        <v>309</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>310</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="72"/>
+      <c r="C8" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D8" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E8" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F8" t="s">
         <v>45</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="47"/>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="F7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="47"/>
-      <c r="C8" s="57" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="68" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" s="59" t="s">
-        <v>143</v>
-      </c>
-      <c r="F8" s="58" t="s">
-        <v>51</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>6</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="72"/>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="72"/>
+      <c r="C10" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J10" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="100" t="s">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="77" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="102" t="s">
+      <c r="C11" s="62" t="s">
         <v>295</v>
       </c>
-      <c r="D9" s="69" t="s">
+      <c r="D11" s="39" t="s">
         <v>297</v>
       </c>
-      <c r="E9" s="103" t="s">
+      <c r="E11" s="63" t="s">
         <v>298</v>
       </c>
-      <c r="F9" s="69" t="s">
+      <c r="F11" s="39" t="s">
         <v>296</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="9" t="s">
+      <c r="G11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="101"/>
-      <c r="C10" s="57" t="s">
+      <c r="J11" s="9"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="78"/>
+      <c r="C12" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="68" t="s">
+      <c r="D12" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="59" t="s">
+      <c r="E12" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="F10" s="58" t="s">
+      <c r="F12" s="32" t="s">
         <v>294</v>
       </c>
-      <c r="G10" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I10" s="9" t="s">
+      <c r="G12" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I12" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J12" s="9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="72" t="s">
         <v>84</v>
       </c>
-      <c r="C11" s="92" t="s">
+      <c r="C13" s="55" t="s">
         <v>85</v>
       </c>
-      <c r="D11" s="78" t="s">
+      <c r="D13" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="87" t="s">
+      <c r="E13" s="50" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="77" t="s">
+      <c r="F13" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="9" t="s">
+      <c r="G13" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I13" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J13" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="47"/>
-      <c r="C12" s="57" t="s">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="72"/>
+      <c r="C14" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D12" s="68" t="s">
+      <c r="D14" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="59" t="s">
+      <c r="E14" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="58" t="s">
+      <c r="F14" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I14" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="J14" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="47" t="s">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="72" t="s">
         <v>93</v>
       </c>
-      <c r="C13" s="69" t="s">
+      <c r="C15" s="39" t="s">
         <v>286</v>
       </c>
-      <c r="D13" s="70" t="s">
+      <c r="D15" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E13" s="71"/>
-      <c r="F13" s="69" t="s">
+      <c r="E15" s="41"/>
+      <c r="F15" s="39" t="s">
         <v>285</v>
       </c>
-      <c r="G13" s="6"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9" t="s">
+      <c r="G15" s="6"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="47"/>
-      <c r="C14" s="69" t="s">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="72"/>
+      <c r="C16" s="39" t="s">
         <v>283</v>
       </c>
-      <c r="D14" s="70" t="s">
+      <c r="D16" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E14" s="71"/>
-      <c r="F14" s="69" t="s">
+      <c r="E16" s="41"/>
+      <c r="F16" s="39" t="s">
         <v>282</v>
       </c>
-      <c r="G14" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9" t="s">
+      <c r="G16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="47"/>
-      <c r="C15" s="69" t="s">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="72"/>
+      <c r="C17" s="39" t="s">
         <v>239</v>
       </c>
-      <c r="D15" s="70" t="s">
+      <c r="D17" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E15" s="71"/>
-      <c r="F15" s="69" t="s">
+      <c r="E17" s="41"/>
+      <c r="F17" s="39" t="s">
         <v>281</v>
       </c>
-      <c r="G15" s="6"/>
-      <c r="I15" s="9" t="s">
+      <c r="G17" s="6"/>
+      <c r="I17" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="47"/>
-      <c r="C16" s="69" t="s">
+      <c r="J17" s="9"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="72"/>
+      <c r="C18" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="70" t="s">
+      <c r="D18" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="E16" s="72"/>
-      <c r="F16" s="69" t="s">
+      <c r="E18" s="42"/>
+      <c r="F18" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I16" s="9" t="s">
+      <c r="G18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="47"/>
-      <c r="C17" s="69" t="s">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="72"/>
+      <c r="C19" s="39" t="s">
         <v>230</v>
       </c>
-      <c r="D17" s="70" t="s">
+      <c r="D19" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="E17" s="72"/>
-      <c r="F17" s="69" t="s">
+      <c r="E19" s="42"/>
+      <c r="F19" s="39" t="s">
         <v>232</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I17" s="9" t="s">
+      <c r="G19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I19" s="9" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="47"/>
-      <c r="C18" s="69" t="s">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="72"/>
+      <c r="C20" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="D18" s="70" t="s">
+      <c r="D20" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="72"/>
-      <c r="F18" s="69" t="s">
+      <c r="E20" s="42"/>
+      <c r="F20" s="39" t="s">
         <v>227</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I18" s="9" t="s">
+      <c r="G20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I20" s="9" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="47"/>
-      <c r="C19" s="69" t="s">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="72"/>
+      <c r="C21" s="39" t="s">
         <v>235</v>
       </c>
-      <c r="D19" s="70" t="s">
+      <c r="D21" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="72"/>
-      <c r="F19" s="69" t="s">
+      <c r="E21" s="42"/>
+      <c r="F21" s="39" t="s">
         <v>228</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I19" s="9" t="s">
+      <c r="G21" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I21" s="9" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="47"/>
-      <c r="C20" s="69" t="s">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="72"/>
+      <c r="C22" s="39" t="s">
         <v>237</v>
       </c>
-      <c r="D20" s="70" t="s">
+      <c r="D22" s="40" t="s">
         <v>95</v>
       </c>
-      <c r="E20" s="72"/>
-      <c r="F20" s="69" t="s">
+      <c r="E22" s="42"/>
+      <c r="F22" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I22" s="9" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="47"/>
-      <c r="C21" s="69" t="s">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="72"/>
+      <c r="C23" s="39" t="s">
         <v>288</v>
       </c>
-      <c r="D21" s="70" t="s">
+      <c r="D23" s="40" t="s">
         <v>289</v>
       </c>
-      <c r="E21" s="72"/>
-      <c r="F21" s="69" t="s">
+      <c r="E23" s="42"/>
+      <c r="F23" s="39" t="s">
         <v>290</v>
       </c>
-      <c r="G21" s="6"/>
-      <c r="I21" s="9" t="s">
+      <c r="G23" s="6"/>
+      <c r="I23" s="9" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="47"/>
-      <c r="C22" s="69" t="s">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="72"/>
+      <c r="C24" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="D22" s="70" t="s">
+      <c r="D24" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="72"/>
-      <c r="F22" s="69" t="s">
+      <c r="E24" s="42"/>
+      <c r="F24" s="39" t="s">
         <v>197</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I22" s="9" t="s">
+      <c r="G24" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I24" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="J22" s="9" t="s">
+      <c r="J24" s="9" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="47"/>
-      <c r="C23" s="69" t="s">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="72"/>
+      <c r="C25" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="D23" s="70" t="s">
+      <c r="D25" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="E23" s="72"/>
-      <c r="F23" s="69" t="s">
+      <c r="E25" s="42"/>
+      <c r="F25" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I23" s="9" t="s">
+      <c r="I25" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="J23" s="9" t="s">
+      <c r="J25" s="9" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" s="47" t="s">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="72" t="s">
         <v>241</v>
       </c>
-      <c r="C24" s="73" t="s">
+      <c r="C26" s="43" t="s">
         <v>249</v>
       </c>
-      <c r="D24" s="74" t="s">
+      <c r="D26" s="44" t="s">
         <v>242</v>
       </c>
-      <c r="E24" s="75"/>
-      <c r="F24" s="76" t="s">
+      <c r="E26" s="45"/>
+      <c r="F26" s="46" t="s">
         <v>250</v>
       </c>
-      <c r="G24" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I24" s="9" t="s">
+      <c r="G26" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I26" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="47"/>
-      <c r="C25" s="77" t="s">
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="72"/>
+      <c r="C27" s="39" t="s">
         <v>252</v>
       </c>
-      <c r="D25" s="78" t="s">
+      <c r="D27" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E25" s="79"/>
-      <c r="F25" s="80" t="s">
+      <c r="E27" s="42"/>
+      <c r="F27" s="47" t="s">
         <v>253</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I25" s="9" t="s">
+      <c r="G27" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I27" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="47"/>
-      <c r="C26" s="69" t="s">
+      <c r="J27" s="9"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="72"/>
+      <c r="C28" s="39" t="s">
         <v>246</v>
       </c>
-      <c r="D26" s="70" t="s">
+      <c r="D28" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E26" s="72"/>
-      <c r="F26" s="69" t="s">
+      <c r="E28" s="42"/>
+      <c r="F28" s="39" t="s">
         <v>248</v>
       </c>
-      <c r="G26" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I26" s="9" t="s">
+      <c r="G28" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I28" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="47"/>
-      <c r="C27" s="69" t="s">
+      <c r="J28" s="9"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="72"/>
+      <c r="C29" s="39" t="s">
         <v>256</v>
       </c>
-      <c r="D27" s="70" t="s">
+      <c r="D29" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E27" s="72"/>
-      <c r="F27" s="81" t="s">
+      <c r="E29" s="42"/>
+      <c r="F29" s="47" t="s">
         <v>255</v>
       </c>
-      <c r="G27" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I27" s="9" t="s">
+      <c r="G29" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I29" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="47"/>
-      <c r="C28" s="69" t="s">
+      <c r="J29" s="9"/>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="72"/>
+      <c r="C30" s="39" t="s">
         <v>243</v>
       </c>
-      <c r="D28" s="70" t="s">
+      <c r="D30" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E28" s="72"/>
-      <c r="F28" s="69" t="s">
+      <c r="E30" s="42"/>
+      <c r="F30" s="39" t="s">
         <v>244</v>
       </c>
-      <c r="G28" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I28" s="9" t="s">
+      <c r="G30" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I30" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="J28" s="9"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="47"/>
-      <c r="C29" s="69" t="s">
+      <c r="J30" s="9"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="72"/>
+      <c r="C31" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="D29" s="70" t="s">
+      <c r="D31" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E29" s="72"/>
-      <c r="F29" s="81" t="s">
+      <c r="E31" s="42"/>
+      <c r="F31" s="47" t="s">
         <v>258</v>
       </c>
-      <c r="G29" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I29" s="9" t="s">
+      <c r="G31" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I31" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="J29" s="9"/>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B30" s="47"/>
-      <c r="C30" s="69" t="s">
+      <c r="J31" s="9"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="72"/>
+      <c r="C32" s="39" t="s">
         <v>262</v>
       </c>
-      <c r="D30" s="70" t="s">
+      <c r="D32" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E30" s="72"/>
-      <c r="F30" s="81" t="s">
+      <c r="E32" s="42"/>
+      <c r="F32" s="47" t="s">
         <v>261</v>
       </c>
-      <c r="G30" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I30" s="9" t="s">
+      <c r="G32" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I32" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="J30" s="9"/>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="47"/>
-      <c r="C31" s="69" t="s">
+      <c r="J32" s="9"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B33" s="72"/>
+      <c r="C33" s="39" t="s">
         <v>265</v>
       </c>
-      <c r="D31" s="70" t="s">
+      <c r="D33" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E31" s="72"/>
-      <c r="F31" s="81" t="s">
+      <c r="E33" s="42"/>
+      <c r="F33" s="47" t="s">
         <v>264</v>
       </c>
-      <c r="G31" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I31" s="9" t="s">
+      <c r="G33" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I33" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="J31" s="9"/>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="47"/>
-      <c r="C32" s="69" t="s">
+      <c r="J33" s="9"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" s="72"/>
+      <c r="C34" s="39" t="s">
         <v>268</v>
       </c>
-      <c r="D32" s="70" t="s">
+      <c r="D34" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E32" s="72"/>
-      <c r="F32" s="81" t="s">
+      <c r="E34" s="42"/>
+      <c r="F34" s="47" t="s">
         <v>267</v>
       </c>
-      <c r="G32" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I32" s="9" t="s">
+      <c r="G34" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I34" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="J32" s="9"/>
-    </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="47"/>
-      <c r="C33" s="69" t="s">
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="72"/>
+      <c r="C35" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D33" s="70" t="s">
+      <c r="D35" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E33" s="72"/>
-      <c r="F33" s="81" t="s">
+      <c r="E35" s="42"/>
+      <c r="F35" s="47" t="s">
         <v>270</v>
       </c>
-      <c r="G33" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I33" s="9" t="s">
+      <c r="G35" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I35" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="J33" s="9"/>
-    </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="47"/>
-      <c r="C34" s="82" t="s">
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" s="72"/>
+      <c r="C36" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D34" s="83" t="s">
+      <c r="D36" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E34" s="84"/>
-      <c r="F34" s="82" t="s">
+      <c r="E36" s="42"/>
+      <c r="F36" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="G34" s="6" t="s">
+      <c r="G36" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I34" s="9" t="s">
+      <c r="I36" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="J34" s="9"/>
-    </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="47"/>
-      <c r="C35" s="69" t="s">
+      <c r="J36" s="9"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" s="72"/>
+      <c r="C37" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D35" s="70" t="s">
+      <c r="D37" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E35" s="72"/>
-      <c r="F35" s="81" t="s">
+      <c r="E37" s="42"/>
+      <c r="F37" s="47" t="s">
         <v>276</v>
       </c>
-      <c r="G35" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I35" s="9" t="s">
+      <c r="G37" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I37" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="J35" s="9"/>
-    </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="47"/>
-      <c r="C36" s="69" t="s">
+      <c r="J37" s="9"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B38" s="72"/>
+      <c r="C38" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D36" s="70" t="s">
+      <c r="D38" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="E36" s="72"/>
-      <c r="F36" s="69" t="s">
+      <c r="E38" s="42"/>
+      <c r="F38" s="39" t="s">
         <v>279</v>
       </c>
-      <c r="G36" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I36" s="9" t="s">
+      <c r="G38" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I38" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="J36" s="9"/>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="47"/>
-      <c r="E37" s="24"/>
-      <c r="G37" s="6"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9"/>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="29" t="s">
+      <c r="J38" s="9"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B39" s="72"/>
+      <c r="E39" s="24"/>
+      <c r="G39" s="6"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="29" t="s">
         <v>204</v>
       </c>
-      <c r="C38" s="60" t="s">
+      <c r="C40" s="67" t="s">
         <v>205</v>
       </c>
-      <c r="D38" s="61" t="s">
+      <c r="D40" s="68" t="s">
         <v>207</v>
       </c>
-      <c r="E38" s="62" t="s">
+      <c r="E40" s="69" t="s">
         <v>208</v>
       </c>
-      <c r="F38" s="61" t="s">
+      <c r="F40" s="68" t="s">
         <v>206</v>
       </c>
-      <c r="G38" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I38" s="9" t="s">
+      <c r="G40" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I40" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="J38" s="9" t="s">
+      <c r="J40" s="9" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="47" t="s">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="72" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="63" t="s">
+      <c r="C41" s="64" t="s">
         <v>220</v>
       </c>
-      <c r="D39" s="11" t="s">
+      <c r="D41" s="43" t="s">
         <v>221</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E41" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="F39" s="11" t="s">
+      <c r="F41" s="43" t="s">
         <v>226</v>
       </c>
-      <c r="G39" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I39" s="9" t="s">
+      <c r="G41" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I41" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="J39" s="9" t="s">
+      <c r="J41" s="9" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="47"/>
-      <c r="C40" s="92" t="s">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="72"/>
+      <c r="C42" s="55" t="s">
         <v>164</v>
       </c>
-      <c r="D40" s="78" t="s">
+      <c r="D42" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="E40" s="87" t="s">
+      <c r="E42" s="50" t="s">
         <v>219</v>
       </c>
-      <c r="F40" s="77" t="s">
+      <c r="F42" s="39" t="s">
         <v>222</v>
       </c>
-      <c r="G40" s="6" t="s">
+      <c r="G42" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I42" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B43" s="72"/>
+      <c r="C43" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F43" t="s">
+        <v>105</v>
+      </c>
+      <c r="G43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I40" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="J40" s="9" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B41" s="47"/>
-      <c r="C41" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41" s="64" t="s">
-        <v>106</v>
-      </c>
-      <c r="E41" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="F41" s="64" t="s">
-        <v>105</v>
-      </c>
-      <c r="G41" s="6" t="s">
+      <c r="I43" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B44" s="72"/>
+      <c r="C44" s="55" t="s">
+        <v>300</v>
+      </c>
+      <c r="D44" s="39" t="s">
+        <v>301</v>
+      </c>
+      <c r="E44" s="50" t="s">
+        <v>302</v>
+      </c>
+      <c r="F44" s="100" t="s">
+        <v>303</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I44" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="J44" s="9"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B45" s="72"/>
+      <c r="C45" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="F45" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="G45" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I41" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="J41" s="9" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="47"/>
-      <c r="C42" s="57" t="s">
-        <v>109</v>
-      </c>
-      <c r="D42" s="58" t="s">
-        <v>113</v>
-      </c>
-      <c r="E42" s="59" t="s">
-        <v>148</v>
-      </c>
-      <c r="F42" s="58" t="s">
-        <v>110</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I42" s="9" t="s">
+      <c r="I45" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="J42" s="9" t="s">
+      <c r="J45" s="9" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B43" s="29" t="s">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="60" t="s">
+      <c r="C46" s="70" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="61" t="s">
+      <c r="D46" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="E43" s="62" t="s">
+      <c r="E46" s="69" t="s">
         <v>149</v>
       </c>
-      <c r="F43" s="65" t="s">
+      <c r="F46" s="71" t="s">
         <v>119</v>
       </c>
-      <c r="G43" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I43" s="9" t="s">
+      <c r="G46" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I46" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="J43" s="9" t="s">
+      <c r="J46" s="9" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="47" t="s">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B47" s="72" t="s">
         <v>152</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C47" t="s">
         <v>153</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D47" t="s">
         <v>154</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E47" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F44" s="21" t="s">
+      <c r="F47" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="G44" s="6" t="s">
+      <c r="G47" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J44" s="9" t="s">
+      <c r="J47" s="9" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="47"/>
-      <c r="C45" s="57" t="s">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B48" s="72"/>
+      <c r="C48" s="62" t="s">
         <v>158</v>
       </c>
-      <c r="D45" s="66" t="s">
+      <c r="D48" s="65" t="s">
         <v>159</v>
       </c>
-      <c r="E45" s="66" t="s">
+      <c r="E48" s="65" t="s">
         <v>160</v>
       </c>
-      <c r="F45" s="58" t="s">
+      <c r="F48" s="66" t="s">
         <v>162</v>
       </c>
-      <c r="G45" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I45" s="9" t="s">
+      <c r="G48" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I48" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="J45" s="9" t="s">
+      <c r="J48" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="56" t="s">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="C46" s="60" t="s">
+      <c r="C49" s="34" t="s">
         <v>213</v>
       </c>
-      <c r="D46" s="67"/>
-      <c r="E46" s="61"/>
-      <c r="F46" s="65"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="35"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="6" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B47:B48"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B5:B10"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="B24:B37"/>
-    <mergeCell ref="B13:B23"/>
-    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B41:B45"/>
+    <mergeCell ref="B26:B39"/>
+    <mergeCell ref="B15:B25"/>
+    <mergeCell ref="B11:B12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G5:H9 G10:G45">
+  <conditionalFormatting sqref="G5:H11 G12:G49">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"no"</formula>
     </cfRule>
@@ -3440,86 +3543,93 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:H9 G10:G45" xr:uid="{16E70C10-E0D8-4840-AEA1-7AA8C21C6052}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:H11 G12:G49" xr:uid="{16E70C10-E0D8-4840-AEA1-7AA8C21C6052}">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="J5" r:id="rId1" xr:uid="{77CE8013-1BB1-433D-94A3-B2FAB9921B3A}"/>
     <hyperlink ref="E5" r:id="rId2" xr:uid="{8E84968F-3D5A-40EC-B9C0-E90712451C7F}"/>
-    <hyperlink ref="J6" r:id="rId3" xr:uid="{02A83B75-9123-4893-B449-D8856F7C48B0}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{0A4DBF73-37BE-43D1-86F6-08A54E4D5A74}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{9CE94A8C-34F6-4260-B969-573D2A245667}"/>
-    <hyperlink ref="J7" r:id="rId6" xr:uid="{F1AF7B01-8EF8-4D45-AD7F-F00C9B1E0E4A}"/>
-    <hyperlink ref="I7" r:id="rId7" xr:uid="{0B05A3A8-0A0A-4446-9677-394031162275}"/>
-    <hyperlink ref="J8" r:id="rId8" xr:uid="{523C57AE-A327-42AA-8E99-8F06A162D325}"/>
-    <hyperlink ref="I10" r:id="rId9" xr:uid="{91D0E0B7-7B95-48BC-A721-F3BADC2E68D5}"/>
-    <hyperlink ref="J10" r:id="rId10" xr:uid="{3B705498-1050-4B6F-813A-9E89D27111EC}"/>
-    <hyperlink ref="E10" r:id="rId11" xr:uid="{691A8FF3-0680-401C-A5BB-CA72E59A6F7B}"/>
-    <hyperlink ref="I11" r:id="rId12" xr:uid="{7D3C1811-6BD9-43E5-AF37-933D4003306E}"/>
-    <hyperlink ref="I12" r:id="rId13" xr:uid="{8F53AC38-352C-4657-A4A8-1DE7749D8332}"/>
-    <hyperlink ref="J12" r:id="rId14" xr:uid="{218DA976-742E-4846-AF26-57B1BE9B2D28}"/>
-    <hyperlink ref="E11" r:id="rId15" xr:uid="{F5BC8CEE-F530-48B2-AEB0-05138F66FE72}"/>
-    <hyperlink ref="E12" r:id="rId16" xr:uid="{2F7D2E1C-572A-40A6-A537-AE8A71A84B92}"/>
-    <hyperlink ref="J11" r:id="rId17" xr:uid="{078108F6-3106-4427-8212-509361A32B23}"/>
-    <hyperlink ref="I16" r:id="rId18" xr:uid="{4B806AB2-B5DE-4DCB-AC21-E51C140EAA6F}"/>
-    <hyperlink ref="E41" r:id="rId19" xr:uid="{B84D1D11-4839-4507-866F-3DB821FC7223}"/>
-    <hyperlink ref="J41" r:id="rId20" xr:uid="{45063706-F8DD-4586-B532-1AF1FFE4D222}"/>
-    <hyperlink ref="I41" r:id="rId21" xr:uid="{D608BFA7-83BF-4D1F-82B5-5A142FAD149B}"/>
-    <hyperlink ref="E42" r:id="rId22" xr:uid="{4E4966D7-5D9C-457C-875C-140C265069B0}"/>
-    <hyperlink ref="J42" r:id="rId23" xr:uid="{2C2D94D1-BDF7-426D-8EFB-1C4770F313BB}"/>
-    <hyperlink ref="I42" r:id="rId24" xr:uid="{E1BC785D-5519-4540-A6B1-C307CDC6A748}"/>
-    <hyperlink ref="J43" r:id="rId25" xr:uid="{FE26BA89-AE20-400E-A204-A1D51563DF5F}"/>
-    <hyperlink ref="I43" r:id="rId26" xr:uid="{4380D086-6180-45C1-9F84-52BBDD26E612}"/>
-    <hyperlink ref="E43" r:id="rId27" xr:uid="{F01D8885-58E5-4152-89A6-1D3EFB41E879}"/>
-    <hyperlink ref="E8" r:id="rId28" xr:uid="{A66C6588-B22D-48F2-A4EC-7D0E46AD60F3}"/>
-    <hyperlink ref="E44" r:id="rId29" xr:uid="{B51B99C6-1910-491D-81A6-E411A3AE7908}"/>
-    <hyperlink ref="J44" r:id="rId30" xr:uid="{D4B2B14F-519C-40B0-AC9E-652A1615F7B2}"/>
-    <hyperlink ref="D45" r:id="rId31" display="https://www.digikey.com.au/en/products/filter/transistors/fets-mosfets/single-fets-mosfets/3-smd-sot-23-3-variant/278?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAJgAYWBWWTkAXQIAHMlBABlSgEtiAcxABfRUA" xr:uid="{427053F7-D1E6-4161-A03E-357918EA99BE}"/>
-    <hyperlink ref="J45" r:id="rId32" xr:uid="{A8094415-9801-4570-832C-C2DE47B8EED0}"/>
-    <hyperlink ref="E45" r:id="rId33" xr:uid="{3300C72A-8FEE-49E7-9F94-26680825DC19}"/>
-    <hyperlink ref="I45" r:id="rId34" xr:uid="{12A90CC8-ABE8-4E1C-B7E9-A039C71E7360}"/>
-    <hyperlink ref="I40" r:id="rId35" xr:uid="{9333B8F5-7A23-4277-901C-C048FA77551E}"/>
-    <hyperlink ref="J40" r:id="rId36" xr:uid="{1F9C453E-8146-4ABB-B0D8-ADC0F74BDFDD}"/>
+    <hyperlink ref="J8" r:id="rId3" xr:uid="{02A83B75-9123-4893-B449-D8856F7C48B0}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{0A4DBF73-37BE-43D1-86F6-08A54E4D5A74}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{9CE94A8C-34F6-4260-B969-573D2A245667}"/>
+    <hyperlink ref="J9" r:id="rId6" xr:uid="{F1AF7B01-8EF8-4D45-AD7F-F00C9B1E0E4A}"/>
+    <hyperlink ref="I9" r:id="rId7" xr:uid="{0B05A3A8-0A0A-4446-9677-394031162275}"/>
+    <hyperlink ref="J10" r:id="rId8" xr:uid="{523C57AE-A327-42AA-8E99-8F06A162D325}"/>
+    <hyperlink ref="I12" r:id="rId9" xr:uid="{91D0E0B7-7B95-48BC-A721-F3BADC2E68D5}"/>
+    <hyperlink ref="J12" r:id="rId10" xr:uid="{3B705498-1050-4B6F-813A-9E89D27111EC}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{691A8FF3-0680-401C-A5BB-CA72E59A6F7B}"/>
+    <hyperlink ref="I13" r:id="rId12" xr:uid="{7D3C1811-6BD9-43E5-AF37-933D4003306E}"/>
+    <hyperlink ref="I14" r:id="rId13" xr:uid="{8F53AC38-352C-4657-A4A8-1DE7749D8332}"/>
+    <hyperlink ref="J14" r:id="rId14" xr:uid="{218DA976-742E-4846-AF26-57B1BE9B2D28}"/>
+    <hyperlink ref="E13" r:id="rId15" xr:uid="{F5BC8CEE-F530-48B2-AEB0-05138F66FE72}"/>
+    <hyperlink ref="E14" r:id="rId16" xr:uid="{2F7D2E1C-572A-40A6-A537-AE8A71A84B92}"/>
+    <hyperlink ref="J13" r:id="rId17" xr:uid="{078108F6-3106-4427-8212-509361A32B23}"/>
+    <hyperlink ref="I18" r:id="rId18" xr:uid="{4B806AB2-B5DE-4DCB-AC21-E51C140EAA6F}"/>
+    <hyperlink ref="E43" r:id="rId19" xr:uid="{B84D1D11-4839-4507-866F-3DB821FC7223}"/>
+    <hyperlink ref="J43" r:id="rId20" xr:uid="{45063706-F8DD-4586-B532-1AF1FFE4D222}"/>
+    <hyperlink ref="I43" r:id="rId21" xr:uid="{D608BFA7-83BF-4D1F-82B5-5A142FAD149B}"/>
+    <hyperlink ref="E45" r:id="rId22" xr:uid="{4E4966D7-5D9C-457C-875C-140C265069B0}"/>
+    <hyperlink ref="J45" r:id="rId23" xr:uid="{2C2D94D1-BDF7-426D-8EFB-1C4770F313BB}"/>
+    <hyperlink ref="I45" r:id="rId24" xr:uid="{E1BC785D-5519-4540-A6B1-C307CDC6A748}"/>
+    <hyperlink ref="J46" r:id="rId25" xr:uid="{FE26BA89-AE20-400E-A204-A1D51563DF5F}"/>
+    <hyperlink ref="I46" r:id="rId26" xr:uid="{4380D086-6180-45C1-9F84-52BBDD26E612}"/>
+    <hyperlink ref="E46" r:id="rId27" xr:uid="{F01D8885-58E5-4152-89A6-1D3EFB41E879}"/>
+    <hyperlink ref="E10" r:id="rId28" xr:uid="{A66C6588-B22D-48F2-A4EC-7D0E46AD60F3}"/>
+    <hyperlink ref="E47" r:id="rId29" xr:uid="{B51B99C6-1910-491D-81A6-E411A3AE7908}"/>
+    <hyperlink ref="J47" r:id="rId30" xr:uid="{D4B2B14F-519C-40B0-AC9E-652A1615F7B2}"/>
+    <hyperlink ref="D48" r:id="rId31" display="https://www.digikey.com.au/en/products/filter/transistors/fets-mosfets/single-fets-mosfets/3-smd-sot-23-3-variant/278?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAJgAYWBWWTkAXQIAHMlBABlSgEtiAcxABfRUA" xr:uid="{427053F7-D1E6-4161-A03E-357918EA99BE}"/>
+    <hyperlink ref="J48" r:id="rId32" xr:uid="{A8094415-9801-4570-832C-C2DE47B8EED0}"/>
+    <hyperlink ref="E48" r:id="rId33" xr:uid="{3300C72A-8FEE-49E7-9F94-26680825DC19}"/>
+    <hyperlink ref="I48" r:id="rId34" xr:uid="{12A90CC8-ABE8-4E1C-B7E9-A039C71E7360}"/>
+    <hyperlink ref="I42" r:id="rId35" xr:uid="{9333B8F5-7A23-4277-901C-C048FA77551E}"/>
+    <hyperlink ref="J42" r:id="rId36" xr:uid="{1F9C453E-8146-4ABB-B0D8-ADC0F74BDFDD}"/>
     <hyperlink ref="I5" r:id="rId37" xr:uid="{C4E7B030-4D65-46DD-B8CD-32E254C3E9BC}"/>
-    <hyperlink ref="J22" r:id="rId38" xr:uid="{A2D551F1-2E4B-4156-B207-EC4CE5E7FC8B}"/>
-    <hyperlink ref="I22" r:id="rId39" xr:uid="{CFFF530B-2773-42DF-90C4-202FCF4E4B7A}"/>
-    <hyperlink ref="J23" r:id="rId40" xr:uid="{1FE24F0A-8C01-411C-8F0E-9B469A2CCDEB}"/>
-    <hyperlink ref="I23" r:id="rId41" xr:uid="{E0602950-D812-4F35-BDE3-248BB4726456}"/>
-    <hyperlink ref="E38" r:id="rId42" xr:uid="{B36D8326-BCC3-4582-9004-FC7C01706DCB}"/>
-    <hyperlink ref="J38" r:id="rId43" xr:uid="{30D79133-F02A-453B-AB7E-C10F953868B8}"/>
-    <hyperlink ref="I38" r:id="rId44" xr:uid="{828B557D-59E0-4E1C-B749-5FDFC6187973}"/>
-    <hyperlink ref="E40" r:id="rId45" xr:uid="{17EC64C7-81E0-4782-83D8-B81B200B35F9}"/>
-    <hyperlink ref="E39" r:id="rId46" xr:uid="{CC3FB449-A5FB-45C6-B6EE-0F3148FD427A}"/>
-    <hyperlink ref="J39" r:id="rId47" xr:uid="{03F4CC3D-F7CE-4EE4-A6FB-D01FDB9B37EE}"/>
-    <hyperlink ref="I39" r:id="rId48" xr:uid="{D880243D-A403-4FCF-9CC6-F7F21A6C9531}"/>
-    <hyperlink ref="I17" r:id="rId49" xr:uid="{70F73E41-DF07-46C4-923C-B09B1549CD2A}"/>
-    <hyperlink ref="I18" r:id="rId50" xr:uid="{CD6B6DB7-7493-4EF2-98A9-A90EE48951BD}"/>
-    <hyperlink ref="I19" r:id="rId51" xr:uid="{6622E1FC-21E2-43E6-B4AC-1EF122E0B3F7}"/>
-    <hyperlink ref="I20" r:id="rId52" xr:uid="{1723F688-3A1D-43B1-AC3B-499F0C426F7B}"/>
-    <hyperlink ref="I15" r:id="rId53" xr:uid="{A81A9CF4-EAE7-4735-A627-120A5ECBC244}"/>
-    <hyperlink ref="I36" r:id="rId54" xr:uid="{EE0E96B7-D0BF-4E1B-9B17-8F0AEFB3AB67}"/>
-    <hyperlink ref="I34" r:id="rId55" xr:uid="{491602FF-2002-40B0-8734-1F671A3D275C}"/>
-    <hyperlink ref="I28" r:id="rId56" xr:uid="{4F1B335D-A4E4-456D-BE8B-FDDDC0F528B9}"/>
-    <hyperlink ref="I26" r:id="rId57" xr:uid="{9EA762D5-8683-4FDC-88A0-AD8881169E2A}"/>
-    <hyperlink ref="I24" r:id="rId58" xr:uid="{4BEA9118-C774-4639-B13C-D389B1536CB5}"/>
-    <hyperlink ref="I25" r:id="rId59" xr:uid="{2866869F-7CDB-4FE9-83C4-9B885E101CAE}"/>
-    <hyperlink ref="I27" r:id="rId60" xr:uid="{B453E5C2-522B-43E9-9B83-2257FF7B0411}"/>
-    <hyperlink ref="I29" r:id="rId61" xr:uid="{E58E8250-744D-4652-8731-FF1922BCACFC}"/>
-    <hyperlink ref="I30" r:id="rId62" xr:uid="{69A48636-6644-4631-9727-1A18CAB04886}"/>
-    <hyperlink ref="I31" r:id="rId63" xr:uid="{B007C36B-A8E7-4553-A135-C95A4A3045E4}"/>
-    <hyperlink ref="I32" r:id="rId64" xr:uid="{6DFE29A5-EEA1-4879-A28B-F475821524E8}"/>
-    <hyperlink ref="I33" r:id="rId65" xr:uid="{6AB3DCD0-713D-46CF-A65F-71A21C2CA861}"/>
-    <hyperlink ref="I35" r:id="rId66" xr:uid="{E31DB478-A8CF-4ECF-82D2-365056D7E08A}"/>
-    <hyperlink ref="J14" r:id="rId67" xr:uid="{2123C418-0A72-462C-8A8A-A91BA1AF54EA}"/>
-    <hyperlink ref="J13" r:id="rId68" xr:uid="{198CD9AC-8EDF-4727-951A-CF56D6A99009}"/>
-    <hyperlink ref="I21" r:id="rId69" xr:uid="{D06154EA-5988-42CB-A0CB-7E75E3CABDC0}"/>
-    <hyperlink ref="E9" r:id="rId70" xr:uid="{54E1429C-5566-4D58-A48A-782EFE638B13}"/>
-    <hyperlink ref="I9" r:id="rId71" xr:uid="{ED01D9AA-1992-4051-A318-6F17035B091F}"/>
+    <hyperlink ref="J24" r:id="rId38" xr:uid="{A2D551F1-2E4B-4156-B207-EC4CE5E7FC8B}"/>
+    <hyperlink ref="I24" r:id="rId39" xr:uid="{CFFF530B-2773-42DF-90C4-202FCF4E4B7A}"/>
+    <hyperlink ref="J25" r:id="rId40" xr:uid="{1FE24F0A-8C01-411C-8F0E-9B469A2CCDEB}"/>
+    <hyperlink ref="I25" r:id="rId41" xr:uid="{E0602950-D812-4F35-BDE3-248BB4726456}"/>
+    <hyperlink ref="E40" r:id="rId42" xr:uid="{B36D8326-BCC3-4582-9004-FC7C01706DCB}"/>
+    <hyperlink ref="J40" r:id="rId43" xr:uid="{30D79133-F02A-453B-AB7E-C10F953868B8}"/>
+    <hyperlink ref="I40" r:id="rId44" xr:uid="{828B557D-59E0-4E1C-B749-5FDFC6187973}"/>
+    <hyperlink ref="E42" r:id="rId45" xr:uid="{17EC64C7-81E0-4782-83D8-B81B200B35F9}"/>
+    <hyperlink ref="E41" r:id="rId46" xr:uid="{CC3FB449-A5FB-45C6-B6EE-0F3148FD427A}"/>
+    <hyperlink ref="J41" r:id="rId47" xr:uid="{03F4CC3D-F7CE-4EE4-A6FB-D01FDB9B37EE}"/>
+    <hyperlink ref="I41" r:id="rId48" xr:uid="{D880243D-A403-4FCF-9CC6-F7F21A6C9531}"/>
+    <hyperlink ref="I19" r:id="rId49" xr:uid="{70F73E41-DF07-46C4-923C-B09B1549CD2A}"/>
+    <hyperlink ref="I20" r:id="rId50" xr:uid="{CD6B6DB7-7493-4EF2-98A9-A90EE48951BD}"/>
+    <hyperlink ref="I21" r:id="rId51" xr:uid="{6622E1FC-21E2-43E6-B4AC-1EF122E0B3F7}"/>
+    <hyperlink ref="I22" r:id="rId52" xr:uid="{1723F688-3A1D-43B1-AC3B-499F0C426F7B}"/>
+    <hyperlink ref="I17" r:id="rId53" xr:uid="{A81A9CF4-EAE7-4735-A627-120A5ECBC244}"/>
+    <hyperlink ref="I38" r:id="rId54" xr:uid="{EE0E96B7-D0BF-4E1B-9B17-8F0AEFB3AB67}"/>
+    <hyperlink ref="I36" r:id="rId55" xr:uid="{491602FF-2002-40B0-8734-1F671A3D275C}"/>
+    <hyperlink ref="I30" r:id="rId56" xr:uid="{4F1B335D-A4E4-456D-BE8B-FDDDC0F528B9}"/>
+    <hyperlink ref="I28" r:id="rId57" xr:uid="{9EA762D5-8683-4FDC-88A0-AD8881169E2A}"/>
+    <hyperlink ref="I26" r:id="rId58" xr:uid="{4BEA9118-C774-4639-B13C-D389B1536CB5}"/>
+    <hyperlink ref="I27" r:id="rId59" xr:uid="{2866869F-7CDB-4FE9-83C4-9B885E101CAE}"/>
+    <hyperlink ref="I29" r:id="rId60" xr:uid="{B453E5C2-522B-43E9-9B83-2257FF7B0411}"/>
+    <hyperlink ref="I31" r:id="rId61" xr:uid="{E58E8250-744D-4652-8731-FF1922BCACFC}"/>
+    <hyperlink ref="I32" r:id="rId62" xr:uid="{69A48636-6644-4631-9727-1A18CAB04886}"/>
+    <hyperlink ref="I33" r:id="rId63" xr:uid="{B007C36B-A8E7-4553-A135-C95A4A3045E4}"/>
+    <hyperlink ref="I34" r:id="rId64" xr:uid="{6DFE29A5-EEA1-4879-A28B-F475821524E8}"/>
+    <hyperlink ref="I35" r:id="rId65" xr:uid="{6AB3DCD0-713D-46CF-A65F-71A21C2CA861}"/>
+    <hyperlink ref="I37" r:id="rId66" xr:uid="{E31DB478-A8CF-4ECF-82D2-365056D7E08A}"/>
+    <hyperlink ref="J16" r:id="rId67" xr:uid="{2123C418-0A72-462C-8A8A-A91BA1AF54EA}"/>
+    <hyperlink ref="J15" r:id="rId68" xr:uid="{198CD9AC-8EDF-4727-951A-CF56D6A99009}"/>
+    <hyperlink ref="I23" r:id="rId69" xr:uid="{D06154EA-5988-42CB-A0CB-7E75E3CABDC0}"/>
+    <hyperlink ref="E11" r:id="rId70" xr:uid="{54E1429C-5566-4D58-A48A-782EFE638B13}"/>
+    <hyperlink ref="I11" r:id="rId71" xr:uid="{ED01D9AA-1992-4051-A318-6F17035B091F}"/>
+    <hyperlink ref="E44" r:id="rId72" xr:uid="{100B7E72-9926-433A-AE57-E8E117203EFC}"/>
+    <hyperlink ref="F44" r:id="rId73" xr:uid="{B04C0F62-4FBB-448E-AD09-6BB081C42E1A}"/>
+    <hyperlink ref="I44" r:id="rId74" xr:uid="{157F98ED-804A-45B7-8DCB-B3A547CA4031}"/>
+    <hyperlink ref="E6" r:id="rId75" xr:uid="{448F1111-8B21-4E73-B986-DC32264FF724}"/>
+    <hyperlink ref="I6" r:id="rId76" xr:uid="{F7B3B305-2100-4542-90BC-8A75AF5F7CFD}"/>
+    <hyperlink ref="E7" r:id="rId77" xr:uid="{E6DE2120-0861-4596-BF6E-251153CD52B8}"/>
+    <hyperlink ref="I7" r:id="rId78" xr:uid="{B96F6C79-203F-43DF-8873-FD02681FB4F2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="D20 D18" numberStoredAsText="1"/>
+    <ignoredError sqref="D22 D20" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3541,29 +3651,29 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="51" t="s">
+      <c r="C2" s="95" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="54"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="31" t="s">
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="32"/>
-      <c r="I2" s="31" t="s">
+      <c r="H2" s="74"/>
+      <c r="I2" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="32"/>
+      <c r="J2" s="74"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
       <c r="D3" s="15" t="s">
         <v>37</v>
       </c>
@@ -3587,19 +3697,19 @@
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="93" t="s">
+      <c r="B4" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="89" t="s">
+      <c r="C4" s="52" t="s">
         <v>292</v>
       </c>
-      <c r="D4" s="89" t="s">
+      <c r="D4" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="90" t="s">
+      <c r="E4" s="53" t="s">
         <v>150</v>
       </c>
-      <c r="F4" s="91" t="s">
+      <c r="F4" s="54" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="6" t="s">
@@ -3619,16 +3729,16 @@
       <c r="B5" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="C5" s="39" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="98" t="s">
+      <c r="D5" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="99" t="s">
+      <c r="E5" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="F5" s="98"/>
+      <c r="F5" s="60"/>
       <c r="G5" s="6" t="s">
         <v>5</v>
       </c>
@@ -3643,19 +3753,19 @@
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="69" t="s">
+      <c r="D6" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="71" t="s">
+      <c r="E6" s="41" t="s">
         <v>151</v>
       </c>
-      <c r="F6" s="69" t="s">
+      <c r="F6" s="39" t="s">
         <v>78</v>
       </c>
       <c r="G6" s="6" t="s">
@@ -3666,7 +3776,7 @@
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="47"/>
+      <c r="B7" s="72"/>
       <c r="C7" t="s">
         <v>77</v>
       </c>
@@ -3687,17 +3797,17 @@
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="47"/>
-      <c r="C8" s="69" t="s">
+      <c r="B8" s="72"/>
+      <c r="C8" s="39" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="71" t="s">
+      <c r="E8" s="41" t="s">
         <v>151</v>
       </c>
-      <c r="F8" s="69" t="s">
+      <c r="F8" s="39" t="s">
         <v>82</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -3708,7 +3818,7 @@
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="47"/>
+      <c r="B9" s="72"/>
       <c r="C9" t="s">
         <v>99</v>
       </c>

</xml_diff>